<commit_message>
feat: define LAC scenarios A, B and C
Register the decision roots A_Calibrated_BAU, B_Optimised_VRE and
C_Target_VRE in the lac setup and its Control sheet, as south_asia.yaml
registers its roots, and add their rule files:
- A: BAU plus a build lock (build_cap_rule.py with cap multiplier 0),
  so generation technologies may build only their planned capacity.
- B: the South Asia B build-cap relaxation and family ceilings on the
  LAC families, with the relaxation dependency on A.
- C: the A lock plus six national renewable share targets from NDCs
  (set_vre_targets.py), expressed as solar PV floors scaled to the
  solved A.
The setup policy build_cap_replaces_workbook_values lets the computed
caps replace the ported BAU build caps. The transmission windows come
from the ported BAU. Every chosen number is an ASSUMPTION in its file.

Tests: compile-only build of A and B; the full solver-free suite.
</commit_message>
<xml_diff>
--- a/areas/lac/inputs/scenarios/OSTRAM_Scenario_Inputs.xlsx
+++ b/areas/lac/inputs/scenarios/OSTRAM_Scenario_Inputs.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,6 +506,66 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>Support scenario: the OSTRAM-LAC BAU model as it stands, with no rule scripts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>A_Calibrated_BAU</t>
+        </is>
+      </c>
+      <c r="B3" t="b">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>build_cap_rule.py</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>The study's Tendencial scenario: BAU plus the build lock to planned generation projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B_Optimised_VRE</t>
+        </is>
+      </c>
+      <c r="B4" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>build_cap_rule.py</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Least cost without targets: South Asia B build-cap relaxation and family ceilings. After its rules, every bound is set to the looser of its own value and that of A_Calibrated_BAU built in the same run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C_Target_VRE</t>
+        </is>
+      </c>
+      <c r="B5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>build_cap_rule.py, set_vre_targets.py</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>The study's NDC scenario: the A settings plus each country's renewable share target, scaled to the solved A_Calibrated_BAU.</t>
         </is>
       </c>
     </row>

</xml_diff>